<commit_message>
feat: add finance rulepack extraction and gap report
</commit_message>
<xml_diff>
--- a/evals/finance-rulepack/rendered.xlsx
+++ b/evals/finance-rulepack/rendered.xlsx
@@ -547,7 +547,7 @@
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>requirements: LE-XM-CN-01
-rules: SOD-SUPPLIER-BANK-PAYMENT, CTRL-DUPLICATE-PAYMENT, INT-BANK-PAYMENT-CALLBACK, OBS-AUDIT-LOG
+rules: SOD-SUPPLIER-BANK-PAYMENT, CTRL-DUPLICATE-PAYMENT, APPROVAL-SUPPLIER-BANK-CHANGE, INT-BANK-PAYMENT-CALLBACK, OBS-AUDIT-LOG
 risks: INC-DUP-PAYMENT-PLACEHOLDER
 test_points: TP-RULEPACK-001</t>
         </is>
@@ -561,7 +561,7 @@
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>name: rulepack_refs
-value: SOD-SUPPLIER-BANK-PAYMENT, CTRL-DUPLICATE-PAYMENT, INT-BANK-PAYMENT-CALLBACK, OBS-AUDIT-LOG
+value: SOD-SUPPLIER-BANK-PAYMENT, APPROVAL-SUPPLIER-BANK-CHANGE, CTRL-DUPLICATE-PAYMENT, INT-BANK-PAYMENT-CALLBACK, OBS-AUDIT-LOG
 source: sample_rulepack.json</t>
         </is>
       </c>

</xml_diff>